<commit_message>
atualizando funcoes e relatorio
</commit_message>
<xml_diff>
--- a/datasets/rbf_metricas.xlsx
+++ b/datasets/rbf_metricas.xlsx
@@ -429,7 +429,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>RMSE Final</t>
+          <t>EQM Final</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -493,7 +493,7 @@
         <v>348</v>
       </c>
       <c r="C2" t="n">
-        <v>0.486907</v>
+        <v>0.23707859</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
@@ -533,10 +533,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C3" t="n">
-        <v>0.486907</v>
+        <v>0.23707866</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
@@ -576,10 +576,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C4" t="n">
-        <v>0.486907</v>
+        <v>0.23707861</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C5" t="n">
-        <v>0.486907</v>
+        <v>0.23707865</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -662,10 +662,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C6" t="n">
-        <v>0.486907</v>
+        <v>0.23707857</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
ajustes na formula da variancia
</commit_message>
<xml_diff>
--- a/datasets/rbf_metricas.xlsx
+++ b/datasets/rbf_metricas.xlsx
@@ -490,40 +490,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>348</v>
+        <v>239</v>
       </c>
       <c r="C2" t="n">
-        <v>0.23707859</v>
+        <v>0.12244239</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="n">
-        <v>2</v>
-      </c>
       <c r="H2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
+        <v>90</v>
+      </c>
+      <c r="K2" t="n">
+        <v>100</v>
+      </c>
+      <c r="L2" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="M2" t="n">
         <v>80</v>
-      </c>
-      <c r="K2" t="n">
-        <v>50</v>
-      </c>
-      <c r="L2" t="n">
-        <v>100</v>
-      </c>
-      <c r="M2" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -533,40 +533,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>346</v>
+        <v>238</v>
       </c>
       <c r="C3" t="n">
-        <v>0.23707866</v>
+        <v>0.12244233</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="G3" t="n">
-        <v>2</v>
-      </c>
       <c r="H3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
+        <v>90</v>
+      </c>
+      <c r="K3" t="n">
+        <v>100</v>
+      </c>
+      <c r="L3" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="M3" t="n">
         <v>80</v>
-      </c>
-      <c r="K3" t="n">
-        <v>50</v>
-      </c>
-      <c r="L3" t="n">
-        <v>100</v>
-      </c>
-      <c r="M3" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="4">
@@ -576,40 +576,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>348</v>
+        <v>239</v>
       </c>
       <c r="C4" t="n">
-        <v>0.23707861</v>
+        <v>0.12244236</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="G4" t="n">
-        <v>2</v>
-      </c>
       <c r="H4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" t="n">
+        <v>90</v>
+      </c>
+      <c r="K4" t="n">
+        <v>100</v>
+      </c>
+      <c r="L4" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="M4" t="n">
         <v>80</v>
-      </c>
-      <c r="K4" t="n">
-        <v>50</v>
-      </c>
-      <c r="L4" t="n">
-        <v>100</v>
-      </c>
-      <c r="M4" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -619,40 +619,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>346</v>
+        <v>240</v>
       </c>
       <c r="C5" t="n">
-        <v>0.23707865</v>
+        <v>0.12244233</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="G5" t="n">
-        <v>2</v>
-      </c>
       <c r="H5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
+        <v>90</v>
+      </c>
+      <c r="K5" t="n">
+        <v>100</v>
+      </c>
+      <c r="L5" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="M5" t="n">
         <v>80</v>
-      </c>
-      <c r="K5" t="n">
-        <v>50</v>
-      </c>
-      <c r="L5" t="n">
-        <v>100</v>
-      </c>
-      <c r="M5" t="n">
-        <v>100</v>
       </c>
     </row>
     <row r="6">
@@ -662,40 +662,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>347</v>
+        <v>239</v>
       </c>
       <c r="C6" t="n">
-        <v>0.23707857</v>
+        <v>0.1224424</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
         <v>0</v>
       </c>
-      <c r="G6" t="n">
-        <v>2</v>
-      </c>
       <c r="H6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" t="n">
+        <v>90</v>
+      </c>
+      <c r="K6" t="n">
+        <v>100</v>
+      </c>
+      <c r="L6" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="M6" t="n">
         <v>80</v>
-      </c>
-      <c r="K6" t="n">
-        <v>50</v>
-      </c>
-      <c r="L6" t="n">
-        <v>100</v>
-      </c>
-      <c r="M6" t="n">
-        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>